<commit_message>
style: update UI components and global asset configuration
</commit_message>
<xml_diff>
--- a/public/templates/phases.xlsx
+++ b/public/templates/phases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp1\htdocs\uwz\uwz\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mundia\projects\lms\uwezo-loan-tracking\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFA5BD9-F5DB-4BCB-AD48-B46225395C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9F4419-F0E8-48F6-9BBF-F9C0244D39BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{8435F349-78B3-4C91-8500-E3C6606C5808}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{8435F349-78B3-4C91-8500-E3C6606C5808}"/>
   </bookViews>
   <sheets>
     <sheet name="loan_phases" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <t>S/No.</t>
   </si>
   <si>
-    <t>Phase*</t>
+    <t>Phase Name*</t>
   </si>
 </sst>
 </file>
@@ -129,9 +129,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -169,7 +169,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -275,7 +275,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -417,7 +417,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -426,12 +426,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A22AF0A1-1B72-41A4-A4BF-F78BB7E8D7E7}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="6.81640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -439,23 +440,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="2"/>
       <c r="B2" s="3"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="2"/>
       <c r="B3" s="3"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" s="2"/>
       <c r="B4" s="3"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" s="2"/>
       <c r="B5" s="3"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" s="2"/>
       <c r="B6" s="3"/>
     </row>

</xml_diff>